<commit_message>
Update detection Excel files for performance testing in version 2.4.2
</commit_message>
<xml_diff>
--- a/tests/perf_v2/perf_history/v2.4.2/detection/DETECTION-high-level-summary.xlsx
+++ b/tests/perf_v2/perf_history/v2.4.2/detection/DETECTION-high-level-summary.xlsx
@@ -647,112 +647,112 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>63.8545</v>
+        <v>63.1</v>
       </c>
       <c r="E2" t="n">
-        <v>25.9068</v>
+        <v>25.3174</v>
       </c>
       <c r="F2" t="n">
-        <v>420.1616</v>
+        <v>443.6908</v>
       </c>
       <c r="G2" t="n">
-        <v>925.4459000000001</v>
+        <v>890.5824</v>
       </c>
       <c r="H2" t="n">
-        <v>6.7355</v>
+        <v>6.7573</v>
       </c>
       <c r="I2" t="n">
-        <v>0.3035</v>
+        <v>0.3063</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1436</v>
+        <v>0.1715</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0687</v>
+        <v>0.1142</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6388</v>
+        <v>0.6556999999999999</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1754</v>
+        <v>0.177</v>
       </c>
       <c r="N2" t="n">
-        <v>0.5327</v>
+        <v>0.5632</v>
       </c>
       <c r="O2" t="n">
-        <v>0.1879</v>
+        <v>0.2066</v>
       </c>
       <c r="P2" t="n">
-        <v>1.7502</v>
+        <v>2.3013</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.6965</v>
+        <v>1.2846</v>
       </c>
       <c r="R2" t="n">
-        <v>0.1127</v>
+        <v>0.1319</v>
       </c>
       <c r="S2" t="n">
-        <v>0.0451</v>
+        <v>0.07729999999999999</v>
       </c>
       <c r="T2" t="n">
-        <v>8.5327</v>
+        <v>9.3353</v>
       </c>
       <c r="U2" t="n">
-        <v>5.3204</v>
+        <v>5.7552</v>
       </c>
       <c r="V2" t="n">
-        <v>0.5329</v>
+        <v>0.5633</v>
       </c>
       <c r="W2" t="n">
-        <v>0.1875</v>
+        <v>0.2062</v>
       </c>
       <c r="X2" t="n">
-        <v>0.1248</v>
+        <v>0.1397</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.049</v>
+        <v>0.0684</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.0422</v>
+        <v>0.0467</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.0133</v>
+        <v>0.0198</v>
       </c>
       <c r="AB2" t="n">
-        <v>3.4077</v>
+        <v>3.5494</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.4343</v>
+        <v>2.3772</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.5318000000000001</v>
+        <v>0.5623</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.1859</v>
+        <v>0.2051</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.3764</v>
+        <v>1.9819</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.8776</v>
+        <v>1.4639</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.115</v>
+        <v>0.1334</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.05</v>
+        <v>0.078</v>
       </c>
       <c r="AJ2" t="n">
-        <v>8.4468</v>
+        <v>9.226800000000001</v>
       </c>
       <c r="AK2" t="n">
-        <v>4.9925</v>
+        <v>5.4426</v>
       </c>
       <c r="AL2" t="n">
-        <v>35.6463</v>
+        <v>38.623</v>
       </c>
       <c r="AM2" t="n">
-        <v>32.4924</v>
+        <v>32.6411</v>
       </c>
       <c r="AN2" t="inlineStr">
         <is>
@@ -777,112 +777,112 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>49.3636</v>
+        <v>49.1667</v>
       </c>
       <c r="E3" t="n">
-        <v>18.7985</v>
+        <v>18.1091</v>
       </c>
       <c r="F3" t="n">
-        <v>761.1985</v>
+        <v>764.6015</v>
       </c>
       <c r="G3" t="n">
-        <v>1725.2891</v>
+        <v>1650.9248</v>
       </c>
       <c r="H3" t="n">
-        <v>9.512</v>
+        <v>9.5382</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2357</v>
+        <v>0.2423</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2863</v>
+        <v>0.2874</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0212</v>
+        <v>0.0206</v>
       </c>
       <c r="L3" t="n">
-        <v>0.6788</v>
+        <v>0.6945</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1666</v>
+        <v>0.1679</v>
       </c>
       <c r="N3" t="n">
-        <v>0.5547</v>
+        <v>0.5845</v>
       </c>
       <c r="O3" t="n">
-        <v>0.1804</v>
+        <v>0.1994</v>
       </c>
       <c r="P3" t="n">
-        <v>20.0624</v>
+        <v>20.5393</v>
       </c>
       <c r="Q3" t="n">
-        <v>3.5372</v>
+        <v>3.2944</v>
       </c>
       <c r="R3" t="n">
-        <v>0.4967</v>
+        <v>0.5125999999999999</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0457</v>
+        <v>0.0688</v>
       </c>
       <c r="T3" t="n">
-        <v>42.7936</v>
+        <v>42.2632</v>
       </c>
       <c r="U3" t="n">
-        <v>32.7405</v>
+        <v>31.3727</v>
       </c>
       <c r="V3" t="n">
-        <v>0.555</v>
+        <v>0.5848</v>
       </c>
       <c r="W3" t="n">
-        <v>0.1796</v>
+        <v>0.1987</v>
       </c>
       <c r="X3" t="n">
-        <v>0.1126</v>
+        <v>0.1155</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.0022</v>
+        <v>0.01</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.0993</v>
+        <v>0.102</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.0303</v>
+        <v>0.0305</v>
       </c>
       <c r="AB3" t="n">
-        <v>7.2904</v>
+        <v>7.2679</v>
       </c>
       <c r="AC3" t="n">
-        <v>3.5511</v>
+        <v>3.3997</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.5533</v>
+        <v>0.583</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.1764</v>
+        <v>0.1959</v>
       </c>
       <c r="AF3" t="n">
-        <v>4.7582</v>
+        <v>5.0718</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.7873</v>
+        <v>0.9502</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.1976</v>
+        <v>0.2127</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.0485</v>
+        <v>0.0688</v>
       </c>
       <c r="AJ3" t="n">
-        <v>15.5558</v>
+        <v>15.9367</v>
       </c>
       <c r="AK3" t="n">
-        <v>9.5739</v>
+        <v>9.2478</v>
       </c>
       <c r="AL3" t="n">
-        <v>217.6476</v>
+        <v>233.3771</v>
       </c>
       <c r="AM3" t="n">
-        <v>223.5116</v>
+        <v>220.687</v>
       </c>
       <c r="AN3" t="inlineStr">
         <is>
@@ -907,112 +907,112 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>56.18</v>
+        <v>54.2909</v>
       </c>
       <c r="E4" t="n">
-        <v>18.8633</v>
+        <v>19.2081</v>
       </c>
       <c r="F4" t="n">
-        <v>593.3518</v>
+        <v>826.2112</v>
       </c>
       <c r="G4" t="n">
-        <v>662.2104</v>
+        <v>1013.0982</v>
       </c>
       <c r="H4" t="n">
-        <v>15.3606</v>
+        <v>15.7265</v>
       </c>
       <c r="I4" t="n">
-        <v>1.7542</v>
+        <v>2.0437</v>
       </c>
       <c r="J4" t="n">
-        <v>0.576</v>
+        <v>0.7968</v>
       </c>
       <c r="K4" t="n">
-        <v>0.521</v>
+        <v>0.8619</v>
       </c>
       <c r="L4" t="n">
-        <v>0.7179</v>
+        <v>0.7331</v>
       </c>
       <c r="M4" t="n">
-        <v>0.14</v>
+        <v>0.1439</v>
       </c>
       <c r="N4" t="n">
-        <v>0.5996</v>
+        <v>0.6277</v>
       </c>
       <c r="O4" t="n">
-        <v>0.1693</v>
+        <v>0.1858</v>
       </c>
       <c r="P4" t="n">
-        <v>5.6837</v>
+        <v>6.1578</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.7854</v>
+        <v>1.0839</v>
       </c>
       <c r="R4" t="n">
-        <v>0.2434</v>
+        <v>0.2637</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0501</v>
+        <v>0.0805</v>
       </c>
       <c r="T4" t="n">
-        <v>15.7414</v>
+        <v>16.5588</v>
       </c>
       <c r="U4" t="n">
-        <v>6.7024</v>
+        <v>6.8971</v>
       </c>
       <c r="V4" t="n">
-        <v>0.5997</v>
+        <v>0.6277</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1707</v>
+        <v>0.1868</v>
       </c>
       <c r="X4" t="n">
-        <v>0.1642</v>
+        <v>0.1933</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.09569999999999999</v>
+        <v>0.1302</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.094</v>
+        <v>0.1016</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.0316</v>
+        <v>0.0387</v>
       </c>
       <c r="AB4" t="n">
-        <v>5.8336</v>
+        <v>6.1584</v>
       </c>
       <c r="AC4" t="n">
-        <v>2.802</v>
+        <v>2.8644</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.4365</v>
+        <v>0.4652</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.2909</v>
+        <v>0.3135</v>
       </c>
       <c r="AF4" t="n">
-        <v>2.5575</v>
+        <v>3.2175</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.7457</v>
+        <v>1.3396</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.221</v>
+        <v>0.2404</v>
       </c>
       <c r="AI4" t="n">
-        <v>0.0673</v>
+        <v>0.0892</v>
       </c>
       <c r="AJ4" t="n">
-        <v>13.6203</v>
+        <v>14.4729</v>
       </c>
       <c r="AK4" t="n">
-        <v>5.174</v>
+        <v>5.6369</v>
       </c>
       <c r="AL4" t="n">
-        <v>251.9585</v>
+        <v>288.0949</v>
       </c>
       <c r="AM4" t="n">
-        <v>295.4298</v>
+        <v>304.2931</v>
       </c>
       <c r="AN4" t="inlineStr">
         <is>
@@ -1037,112 +1037,112 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>49.6727</v>
+        <v>49</v>
       </c>
       <c r="E5" t="n">
-        <v>13.1882</v>
+        <v>12.9798</v>
       </c>
       <c r="F5" t="n">
-        <v>1142.8099</v>
+        <v>1455.8141</v>
       </c>
       <c r="G5" t="n">
-        <v>1834.8997</v>
+        <v>2055.5979</v>
       </c>
       <c r="H5" t="n">
-        <v>10.6824</v>
+        <v>10.7663</v>
       </c>
       <c r="I5" t="n">
-        <v>2.2832</v>
+        <v>2.2043</v>
       </c>
       <c r="J5" t="n">
-        <v>0.4726</v>
+        <v>0.6348</v>
       </c>
       <c r="K5" t="n">
-        <v>0.3599</v>
+        <v>0.6429</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6623</v>
+        <v>0.6849</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1739</v>
+        <v>0.1827</v>
       </c>
       <c r="N5" t="n">
-        <v>0.5391</v>
+        <v>0.5733</v>
       </c>
       <c r="O5" t="n">
-        <v>0.2153</v>
+        <v>0.2357</v>
       </c>
       <c r="P5" t="n">
-        <v>7.8609</v>
+        <v>8.098699999999999</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.3459</v>
+        <v>1.2986</v>
       </c>
       <c r="R5" t="n">
-        <v>0.2606</v>
+        <v>0.2792</v>
       </c>
       <c r="S5" t="n">
-        <v>0.0493</v>
+        <v>0.0784</v>
       </c>
       <c r="T5" t="n">
-        <v>21.6435</v>
+        <v>21.9796</v>
       </c>
       <c r="U5" t="n">
-        <v>15.4159</v>
+        <v>14.7929</v>
       </c>
       <c r="V5" t="n">
-        <v>0.5411</v>
+        <v>0.5752</v>
       </c>
       <c r="W5" t="n">
-        <v>0.2133</v>
+        <v>0.2337</v>
       </c>
       <c r="X5" t="n">
-        <v>0.1622</v>
+        <v>0.1891</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.0867</v>
+        <v>0.1224</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.1061</v>
+        <v>0.1137</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.0381</v>
+        <v>0.0445</v>
       </c>
       <c r="AB5" t="n">
-        <v>7.7422</v>
+        <v>7.9685</v>
       </c>
       <c r="AC5" t="n">
-        <v>4.0402</v>
+        <v>3.9396</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.4733</v>
+        <v>0.5125999999999999</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.2224</v>
+        <v>0.2503</v>
       </c>
       <c r="AF5" t="n">
-        <v>3.3558</v>
+        <v>3.7608</v>
       </c>
       <c r="AG5" t="n">
-        <v>0.5888</v>
+        <v>0.986</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.206</v>
+        <v>0.223</v>
       </c>
       <c r="AI5" t="n">
-        <v>0.0672</v>
+        <v>0.0859</v>
       </c>
       <c r="AJ5" t="n">
-        <v>15.8479</v>
+        <v>16.3378</v>
       </c>
       <c r="AK5" t="n">
-        <v>9.6957</v>
+        <v>9.4207</v>
       </c>
       <c r="AL5" t="n">
-        <v>119.2972</v>
+        <v>127.4897</v>
       </c>
       <c r="AM5" t="n">
-        <v>93.98560000000001</v>
+        <v>94.0029</v>
       </c>
       <c r="AN5" t="inlineStr">
         <is>
@@ -1167,112 +1167,112 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>55.0909</v>
+        <v>53.3833</v>
       </c>
       <c r="E6" t="n">
-        <v>16.8976</v>
+        <v>17.185</v>
       </c>
       <c r="F6" t="n">
-        <v>1241.4178</v>
+        <v>1521.1801</v>
       </c>
       <c r="G6" t="n">
-        <v>2477.884</v>
+        <v>2553.7721</v>
       </c>
       <c r="H6" t="n">
-        <v>3.904</v>
+        <v>3.9628</v>
       </c>
       <c r="I6" t="n">
-        <v>1.4184</v>
+        <v>1.3753</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4295</v>
+        <v>0.6281</v>
       </c>
       <c r="K6" t="n">
-        <v>0.4397</v>
+        <v>0.7863</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6137</v>
+        <v>0.6329</v>
       </c>
       <c r="M6" t="n">
-        <v>0.1896</v>
+        <v>0.1957</v>
       </c>
       <c r="N6" t="n">
-        <v>0.4777</v>
+        <v>0.5098</v>
       </c>
       <c r="O6" t="n">
-        <v>0.2391</v>
+        <v>0.2553</v>
       </c>
       <c r="P6" t="n">
-        <v>2.1799</v>
+        <v>2.7056</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.5935</v>
+        <v>1.1984</v>
       </c>
       <c r="R6" t="n">
-        <v>0.1244</v>
+        <v>0.1474</v>
       </c>
       <c r="S6" t="n">
-        <v>0.046</v>
+        <v>0.0887</v>
       </c>
       <c r="T6" t="n">
-        <v>9.9658</v>
+        <v>10.9033</v>
       </c>
       <c r="U6" t="n">
-        <v>7.2086</v>
+        <v>7.5801</v>
       </c>
       <c r="V6" t="n">
-        <v>0.4763</v>
+        <v>0.5085</v>
       </c>
       <c r="W6" t="n">
-        <v>0.2408</v>
+        <v>0.257</v>
       </c>
       <c r="X6" t="n">
-        <v>0.1335</v>
+        <v>0.1668</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.1116</v>
+        <v>0.1549</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.0594</v>
+        <v>0.0677</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.0269</v>
+        <v>0.0378</v>
       </c>
       <c r="AB6" t="n">
-        <v>4.824</v>
+        <v>5.1222</v>
       </c>
       <c r="AC6" t="n">
-        <v>3.9754</v>
+        <v>3.9337</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.3852</v>
+        <v>0.4246</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.2451</v>
+        <v>0.2717</v>
       </c>
       <c r="AF6" t="n">
-        <v>1.4752</v>
+        <v>2.0808</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.7745</v>
+        <v>1.4201</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.1301</v>
+        <v>0.149</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.0781</v>
+        <v>0.098</v>
       </c>
       <c r="AJ6" t="n">
-        <v>10.1554</v>
+        <v>10.8867</v>
       </c>
       <c r="AK6" t="n">
-        <v>9.3612</v>
+        <v>9.2842</v>
       </c>
       <c r="AL6" t="n">
-        <v>42.4596</v>
+        <v>46.7</v>
       </c>
       <c r="AM6" t="n">
-        <v>34.906</v>
+        <v>36.2814</v>
       </c>
       <c r="AN6" t="inlineStr">
         <is>
@@ -1297,112 +1297,112 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>48.6545</v>
+        <v>48.2667</v>
       </c>
       <c r="E7" t="n">
-        <v>14.8651</v>
+        <v>15.3599</v>
       </c>
       <c r="F7" t="n">
-        <v>993.0888</v>
+        <v>1372.4138</v>
       </c>
       <c r="G7" t="n">
-        <v>1645.2763</v>
+        <v>2135.01</v>
       </c>
       <c r="H7" t="n">
-        <v>7.8665</v>
+        <v>7.9387</v>
       </c>
       <c r="I7" t="n">
-        <v>2.3201</v>
+        <v>2.2342</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4712</v>
+        <v>0.6525</v>
       </c>
       <c r="K7" t="n">
-        <v>0.3984</v>
+        <v>0.7164</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6559</v>
+        <v>0.6764</v>
       </c>
       <c r="M7" t="n">
-        <v>0.1697</v>
+        <v>0.1768</v>
       </c>
       <c r="N7" t="n">
-        <v>0.5345</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="O7" t="n">
-        <v>0.2127</v>
+        <v>0.231</v>
       </c>
       <c r="P7" t="n">
-        <v>4.1771</v>
+        <v>4.5381</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.6738</v>
+        <v>0.9534</v>
       </c>
       <c r="R7" t="n">
-        <v>0.1805</v>
+        <v>0.1999</v>
       </c>
       <c r="S7" t="n">
-        <v>0.0467</v>
+        <v>0.0788</v>
       </c>
       <c r="T7" t="n">
-        <v>14.5514</v>
+        <v>15.1632</v>
       </c>
       <c r="U7" t="n">
-        <v>9.8574</v>
+        <v>9.6516</v>
       </c>
       <c r="V7" t="n">
-        <v>0.5355</v>
+        <v>0.5677</v>
       </c>
       <c r="W7" t="n">
-        <v>0.2121</v>
+        <v>0.2302</v>
       </c>
       <c r="X7" t="n">
-        <v>0.1454</v>
+        <v>0.1729</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.09719999999999999</v>
+        <v>0.1308</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.0785</v>
+        <v>0.0858</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.0297</v>
+        <v>0.0374</v>
       </c>
       <c r="AB7" t="n">
-        <v>5.9888</v>
+        <v>6.2198</v>
       </c>
       <c r="AC7" t="n">
-        <v>3.9399</v>
+        <v>3.8483</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.4441</v>
+        <v>0.483</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.2406</v>
+        <v>0.2646</v>
       </c>
       <c r="AF7" t="n">
-        <v>2.5831</v>
+        <v>3.0403</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.6221</v>
+        <v>1.0922</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.1736</v>
+        <v>0.1914</v>
       </c>
       <c r="AI7" t="n">
-        <v>0.0584</v>
+        <v>0.08169999999999999</v>
       </c>
       <c r="AJ7" t="n">
-        <v>13.1178</v>
+        <v>13.7355</v>
       </c>
       <c r="AK7" t="n">
-        <v>7.5372</v>
+        <v>7.5014</v>
       </c>
       <c r="AL7" t="n">
-        <v>82.39830000000001</v>
+        <v>88.6972</v>
       </c>
       <c r="AM7" t="n">
-        <v>67.02889999999999</v>
+        <v>67.4983</v>
       </c>
       <c r="AN7" t="inlineStr">
         <is>
@@ -1427,112 +1427,112 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>73.0909</v>
+        <v>73.7667</v>
       </c>
       <c r="E8" t="n">
-        <v>27.5851</v>
+        <v>26.5766</v>
       </c>
       <c r="F8" t="n">
-        <v>647.9431</v>
+        <v>764.846</v>
       </c>
       <c r="G8" t="n">
-        <v>1481.2288</v>
+        <v>1470.9693</v>
       </c>
       <c r="H8" t="n">
-        <v>2.1865</v>
+        <v>2.2008</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6654</v>
+        <v>0.6392</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1512</v>
+        <v>0.2221</v>
       </c>
       <c r="K8" t="n">
-        <v>0.1169</v>
+        <v>0.2623</v>
       </c>
       <c r="L8" t="n">
-        <v>0.6239</v>
+        <v>0.6456</v>
       </c>
       <c r="M8" t="n">
-        <v>0.1834</v>
+        <v>0.1899</v>
       </c>
       <c r="N8" t="n">
-        <v>0.5104</v>
+        <v>0.5452</v>
       </c>
       <c r="O8" t="n">
-        <v>0.1962</v>
+        <v>0.2209</v>
       </c>
       <c r="P8" t="n">
-        <v>1.2223</v>
+        <v>1.8454</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.8011</v>
+        <v>1.4585</v>
       </c>
       <c r="R8" t="n">
-        <v>0.0955</v>
+        <v>0.1172</v>
       </c>
       <c r="S8" t="n">
-        <v>0.0455</v>
+        <v>0.0848</v>
       </c>
       <c r="T8" t="n">
-        <v>7.2675</v>
+        <v>8.236700000000001</v>
       </c>
       <c r="U8" t="n">
-        <v>5.163</v>
+        <v>5.9095</v>
       </c>
       <c r="V8" t="n">
-        <v>0.5118</v>
+        <v>0.5466</v>
       </c>
       <c r="W8" t="n">
-        <v>0.2012</v>
+        <v>0.2249</v>
       </c>
       <c r="X8" t="n">
-        <v>0.1106</v>
+        <v>0.1337</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.0447</v>
+        <v>0.09180000000000001</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.0432</v>
+        <v>0.0491</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.0141</v>
+        <v>0.0243</v>
       </c>
       <c r="AB8" t="n">
-        <v>3.6886</v>
+        <v>3.8842</v>
       </c>
       <c r="AC8" t="n">
-        <v>3.033</v>
+        <v>2.9839</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.5002</v>
+        <v>0.5354</v>
       </c>
       <c r="AE8" t="n">
-        <v>0.1973</v>
+        <v>0.2224</v>
       </c>
       <c r="AF8" t="n">
-        <v>1.1316</v>
+        <v>1.7701</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.8532999999999999</v>
+        <v>1.5106</v>
       </c>
       <c r="AH8" t="n">
-        <v>0.1007</v>
+        <v>0.1197</v>
       </c>
       <c r="AI8" t="n">
-        <v>0.0474</v>
+        <v>0.0781</v>
       </c>
       <c r="AJ8" t="n">
-        <v>7.5559</v>
+        <v>8.378399999999999</v>
       </c>
       <c r="AK8" t="n">
-        <v>5.1346</v>
+        <v>5.6317</v>
       </c>
       <c r="AL8" t="n">
-        <v>20.6398</v>
+        <v>22.337</v>
       </c>
       <c r="AM8" t="n">
-        <v>15.1396</v>
+        <v>15.557</v>
       </c>
       <c r="AN8" t="inlineStr">
         <is>
@@ -1557,112 +1557,112 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>76.7818</v>
+        <v>78.15000000000001</v>
       </c>
       <c r="E9" t="n">
-        <v>26.1213</v>
+        <v>25.7253</v>
       </c>
       <c r="F9" t="n">
-        <v>631.5748</v>
+        <v>820.6477</v>
       </c>
       <c r="G9" t="n">
-        <v>1227.0396</v>
+        <v>1338.5758</v>
       </c>
       <c r="H9" t="n">
-        <v>5.6816</v>
+        <v>5.713</v>
       </c>
       <c r="I9" t="n">
-        <v>0.448</v>
+        <v>0.4442</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1903</v>
+        <v>0.2819</v>
       </c>
       <c r="K9" t="n">
-        <v>0.2357</v>
+        <v>0.3806</v>
       </c>
       <c r="L9" t="n">
-        <v>0.5568</v>
+        <v>0.579</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2005</v>
+        <v>0.2058</v>
       </c>
       <c r="N9" t="n">
-        <v>0.4249</v>
+        <v>0.4617</v>
       </c>
       <c r="O9" t="n">
-        <v>0.214</v>
+        <v>0.2389</v>
       </c>
       <c r="P9" t="n">
-        <v>1.4525</v>
+        <v>2.0282</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.6691</v>
+        <v>1.3177</v>
       </c>
       <c r="R9" t="n">
-        <v>0.0958</v>
+        <v>0.1156</v>
       </c>
       <c r="S9" t="n">
-        <v>0.0437</v>
+        <v>0.07829999999999999</v>
       </c>
       <c r="T9" t="n">
-        <v>7.5759</v>
+        <v>8.4161</v>
       </c>
       <c r="U9" t="n">
-        <v>5.7564</v>
+        <v>6.184</v>
       </c>
       <c r="V9" t="n">
-        <v>0.4247</v>
+        <v>0.4615</v>
       </c>
       <c r="W9" t="n">
-        <v>0.2142</v>
+        <v>0.2391</v>
       </c>
       <c r="X9" t="n">
-        <v>0.1197</v>
+        <v>0.1355</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.0456</v>
+        <v>0.0689</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.043</v>
+        <v>0.048</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.0164</v>
+        <v>0.023</v>
       </c>
       <c r="AB9" t="n">
-        <v>3.6216</v>
+        <v>3.7748</v>
       </c>
       <c r="AC9" t="n">
-        <v>3.0305</v>
+        <v>2.9446</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.4252</v>
+        <v>0.4621</v>
       </c>
       <c r="AE9" t="n">
-        <v>0.214</v>
+        <v>0.2392</v>
       </c>
       <c r="AF9" t="n">
-        <v>1.0915</v>
+        <v>1.7105</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.8578</v>
+        <v>1.4771</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.0902</v>
+        <v>0.1093</v>
       </c>
       <c r="AI9" t="n">
-        <v>0.0486</v>
+        <v>0.0791</v>
       </c>
       <c r="AJ9" t="n">
-        <v>6.984</v>
+        <v>7.8128</v>
       </c>
       <c r="AK9" t="n">
-        <v>5.5278</v>
+        <v>5.9719</v>
       </c>
       <c r="AL9" t="n">
-        <v>26.4151</v>
+        <v>28.9163</v>
       </c>
       <c r="AM9" t="n">
-        <v>26.0555</v>
+        <v>26.2935</v>
       </c>
       <c r="AN9" t="inlineStr">
         <is>
@@ -1687,112 +1687,112 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>63.3273</v>
+        <v>62.3167</v>
       </c>
       <c r="E10" t="n">
-        <v>22.0413</v>
+        <v>21.7283</v>
       </c>
       <c r="F10" t="n">
-        <v>572.0854</v>
+        <v>613.1504</v>
       </c>
       <c r="G10" t="n">
-        <v>1248.7826</v>
+        <v>1205.3464</v>
       </c>
       <c r="H10" t="n">
-        <v>8.042</v>
+        <v>8.065</v>
       </c>
       <c r="I10" t="n">
-        <v>1.3588</v>
+        <v>1.3034</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1735</v>
+        <v>0.2241</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1151</v>
+        <v>0.202</v>
       </c>
       <c r="L10" t="n">
-        <v>0.6623</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>0.1857</v>
+        <v>0.1919</v>
       </c>
       <c r="N10" t="n">
-        <v>0.5475</v>
+        <v>0.5805</v>
       </c>
       <c r="O10" t="n">
-        <v>0.2108</v>
+        <v>0.2299</v>
       </c>
       <c r="P10" t="n">
-        <v>4.3922</v>
+        <v>4.7517</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.7355</v>
+        <v>0.9848</v>
       </c>
       <c r="R10" t="n">
-        <v>0.169</v>
+        <v>0.1874</v>
       </c>
       <c r="S10" t="n">
-        <v>0.0402</v>
+        <v>0.07240000000000001</v>
       </c>
       <c r="T10" t="n">
-        <v>13.8342</v>
+        <v>14.3996</v>
       </c>
       <c r="U10" t="n">
-        <v>9.686199999999999</v>
+        <v>9.4582</v>
       </c>
       <c r="V10" t="n">
-        <v>0.556</v>
+        <v>0.5881</v>
       </c>
       <c r="W10" t="n">
-        <v>0.2178</v>
+        <v>0.2345</v>
       </c>
       <c r="X10" t="n">
-        <v>0.0911</v>
+        <v>0.1059</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.042</v>
+        <v>0.06519999999999999</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.0789</v>
+        <v>0.08359999999999999</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.0307</v>
+        <v>0.0334</v>
       </c>
       <c r="AB10" t="n">
-        <v>5.8235</v>
+        <v>5.9343</v>
       </c>
       <c r="AC10" t="n">
-        <v>3.3736</v>
+        <v>3.2515</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.5448</v>
+        <v>0.5772</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.2126</v>
+        <v>0.2305</v>
       </c>
       <c r="AF10" t="n">
-        <v>1.7659</v>
+        <v>2.3422</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.824</v>
+        <v>1.3865</v>
       </c>
       <c r="AH10" t="n">
-        <v>0.1303</v>
+        <v>0.1491</v>
       </c>
       <c r="AI10" t="n">
-        <v>0.0514</v>
+        <v>0.0798</v>
       </c>
       <c r="AJ10" t="n">
-        <v>9.819900000000001</v>
+        <v>10.5723</v>
       </c>
       <c r="AK10" t="n">
-        <v>6.0425</v>
+        <v>6.3051</v>
       </c>
       <c r="AL10" t="n">
-        <v>56.2505</v>
+        <v>60.1439</v>
       </c>
       <c r="AM10" t="n">
-        <v>43.3644</v>
+        <v>43.4821</v>
       </c>
       <c r="AN10" t="inlineStr">
         <is>
@@ -1817,112 +1817,112 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>72.9636</v>
+        <v>71.3</v>
       </c>
       <c r="E11" t="n">
-        <v>26.5246</v>
+        <v>26.0666</v>
       </c>
       <c r="F11" t="n">
-        <v>529.9664</v>
+        <v>578.0968</v>
       </c>
       <c r="G11" t="n">
-        <v>1195.5122</v>
+        <v>1155.7812</v>
       </c>
       <c r="H11" t="n">
-        <v>3.35</v>
+        <v>3.3973</v>
       </c>
       <c r="I11" t="n">
-        <v>1.728</v>
+        <v>1.6614</v>
       </c>
       <c r="J11" t="n">
-        <v>0.1347</v>
+        <v>0.1912</v>
       </c>
       <c r="K11" t="n">
-        <v>0.1107</v>
+        <v>0.2168</v>
       </c>
       <c r="L11" t="n">
-        <v>0.6373</v>
+        <v>0.6596</v>
       </c>
       <c r="M11" t="n">
-        <v>0.1828</v>
+        <v>0.1901</v>
       </c>
       <c r="N11" t="n">
-        <v>0.5185</v>
+        <v>0.5528</v>
       </c>
       <c r="O11" t="n">
-        <v>0.2155</v>
+        <v>0.236</v>
       </c>
       <c r="P11" t="n">
-        <v>1.3652</v>
+        <v>2.047</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.7847</v>
+        <v>1.5806</v>
       </c>
       <c r="R11" t="n">
-        <v>0.1007</v>
+        <v>0.1224</v>
       </c>
       <c r="S11" t="n">
-        <v>0.0444</v>
+        <v>0.0843</v>
       </c>
       <c r="T11" t="n">
-        <v>7.7601</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="U11" t="n">
-        <v>5.4688</v>
+        <v>6.1264</v>
       </c>
       <c r="V11" t="n">
-        <v>0.5246</v>
+        <v>0.5585</v>
       </c>
       <c r="W11" t="n">
-        <v>0.2222</v>
+        <v>0.241</v>
       </c>
       <c r="X11" t="n">
-        <v>0.0953</v>
+        <v>0.1222</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.0521</v>
+        <v>0.1029</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.0448</v>
+        <v>0.0514</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.021</v>
+        <v>0.0299</v>
       </c>
       <c r="AB11" t="n">
-        <v>3.7089</v>
+        <v>3.9477</v>
       </c>
       <c r="AC11" t="n">
-        <v>3.222</v>
+        <v>3.1855</v>
       </c>
       <c r="AD11" t="n">
-        <v>0.5127</v>
+        <v>0.5465</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.2191</v>
+        <v>0.2382</v>
       </c>
       <c r="AF11" t="n">
-        <v>1.1798</v>
+        <v>1.8556</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.8116</v>
+        <v>1.5742</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.1014</v>
+        <v>0.1214</v>
       </c>
       <c r="AI11" t="n">
-        <v>0.0474</v>
+        <v>0.0809</v>
       </c>
       <c r="AJ11" t="n">
-        <v>7.6689</v>
+        <v>8.5373</v>
       </c>
       <c r="AK11" t="n">
-        <v>5.2745</v>
+        <v>5.8288</v>
       </c>
       <c r="AL11" t="n">
-        <v>23.467</v>
+        <v>25.8271</v>
       </c>
       <c r="AM11" t="n">
-        <v>17.5468</v>
+        <v>18.7342</v>
       </c>
       <c r="AN11" t="inlineStr">
         <is>
@@ -1947,112 +1947,112 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>64.4182</v>
+        <v>64.91670000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>26.1099</v>
+        <v>25.7401</v>
       </c>
       <c r="F12" t="n">
-        <v>366.899</v>
+        <v>428.8596</v>
       </c>
       <c r="G12" t="n">
-        <v>856.0449</v>
+        <v>850.0498</v>
       </c>
       <c r="H12" t="n">
-        <v>2.5189</v>
+        <v>2.5615</v>
       </c>
       <c r="I12" t="n">
-        <v>1.1116</v>
+        <v>1.0751</v>
       </c>
       <c r="J12" t="n">
-        <v>0.1213</v>
+        <v>0.1619</v>
       </c>
       <c r="K12" t="n">
-        <v>0.0931</v>
+        <v>0.1622</v>
       </c>
       <c r="L12" t="n">
-        <v>0.6141</v>
+        <v>0.6233</v>
       </c>
       <c r="M12" t="n">
-        <v>0.1735</v>
+        <v>0.169</v>
       </c>
       <c r="N12" t="n">
-        <v>0.4833</v>
+        <v>0.509</v>
       </c>
       <c r="O12" t="n">
-        <v>0.1704</v>
+        <v>0.1844</v>
       </c>
       <c r="P12" t="n">
-        <v>1.078</v>
+        <v>1.7094</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.8507</v>
+        <v>1.4947</v>
       </c>
       <c r="R12" t="n">
-        <v>0.09379999999999999</v>
+        <v>0.1171</v>
       </c>
       <c r="S12" t="n">
-        <v>0.0476</v>
+        <v>0.0905</v>
       </c>
       <c r="T12" t="n">
-        <v>7.0559</v>
+        <v>8.1204</v>
       </c>
       <c r="U12" t="n">
-        <v>5.0798</v>
+        <v>6.0248</v>
       </c>
       <c r="V12" t="n">
-        <v>0.4848</v>
+        <v>0.5103</v>
       </c>
       <c r="W12" t="n">
-        <v>0.1761</v>
+        <v>0.189</v>
       </c>
       <c r="X12" t="n">
-        <v>0.076</v>
+        <v>0.097</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.0572</v>
+        <v>0.0893</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.0366</v>
+        <v>0.042</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.0172</v>
+        <v>0.0244</v>
       </c>
       <c r="AB12" t="n">
-        <v>2.9009</v>
+        <v>3.1061</v>
       </c>
       <c r="AC12" t="n">
-        <v>2.3185</v>
+        <v>2.3232</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.4815</v>
+        <v>0.5053</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.1713</v>
+        <v>0.1823</v>
       </c>
       <c r="AF12" t="n">
-        <v>1.13</v>
+        <v>1.7797</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.8618</v>
+        <v>1.5334</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.09669999999999999</v>
+        <v>0.1185</v>
       </c>
       <c r="AI12" t="n">
-        <v>0.0474</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="AJ12" t="n">
-        <v>7.1842</v>
+        <v>8.170299999999999</v>
       </c>
       <c r="AK12" t="n">
-        <v>4.8456</v>
+        <v>5.6917</v>
       </c>
       <c r="AL12" t="n">
-        <v>15.7953</v>
+        <v>17.2496</v>
       </c>
       <c r="AM12" t="n">
-        <v>9.4298</v>
+        <v>10.2495</v>
       </c>
       <c r="AN12" t="inlineStr">
         <is>

</xml_diff>